<commit_message>
fix: Tahminlenen_Talep sutun adlari Turkce karaktere donusturuldu
</commit_message>
<xml_diff>
--- a/outputs/Tahminlenen_Talep.xlsx
+++ b/outputs/Tahminlenen_Talep.xlsx
@@ -424,12 +424,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Cikis TM</t>
+          <t>Çıkış TM</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Varis TM</t>
+          <t>Varış TM</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">

</xml_diff>